<commit_message>
Wire Tech Hub roadmap data into Product Board
- Refresh public/generated-roadmaps/Digital_Framework.xlsx so production picks up the new Tech Hub sheet (7 rows; same columns as HVAC LC and Daikin City).
- Add 'Tech Hub' / 'Tech hub' as explicit sheetAliases on the techhub product so the lookup is robust to spacing without relying on whitespace normalization.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/generated-roadmaps/Digital_Framework.xlsx
+++ b/public/generated-roadmaps/Digital_Framework.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="382" documentId="11_B8829BEC0D35621E5980E8117F10043E0821A643" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A0667ED-A88D-6745-97E2-D4FA454891A4}"/>
+  <xr:revisionPtr revIDLastSave="391" documentId="11_B8829BEC0D35621E5980E8117F10043E0821A643" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F851D13C-A926-AF4A-8F8E-6FBDED5DB7E7}"/>
   <bookViews>
-    <workbookView xWindow="17060" yWindow="520" windowWidth="40020" windowHeight="22840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14860" yWindow="3080" windowWidth="40400" windowHeight="23820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="HVAC Learning Campus" sheetId="3" r:id="rId1"/>
-    <sheet name="Daikin City" sheetId="4" r:id="rId2"/>
+    <sheet name="Tech Hub" sheetId="5" r:id="rId1"/>
+    <sheet name="HVAC Learning Campus" sheetId="3" r:id="rId2"/>
+    <sheet name="Daikin City" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="111">
   <si>
     <t>Feature Group</t>
   </si>
@@ -308,6 +309,99 @@
   </si>
   <si>
     <t>No customer compliants</t>
+  </si>
+  <si>
+    <t>Video call feature</t>
+  </si>
+  <si>
+    <t>Introduce a new method for Daikin contractors to connect with the support team by adding a video call request form feature to the Daikin Tech Hub app.</t>
+  </si>
+  <si>
+    <t>This will be great help for evey contactor in the field and every technical service team member and both will save tremendous time once this feature goes LIVE.</t>
+  </si>
+  <si>
+    <t>400-500 calls per year</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Integrating of Technical Service Bulletin with Notification</t>
+  </si>
+  <si>
+    <t>Incorporate the Technical Service Bulletin into the Daikin Tech Hub app and activate notifications for all newly released bulletins.</t>
+  </si>
+  <si>
+    <t>This will greatly support the service team, as Daikin often receives feedback highlighting the need for a dedicated, easily accessible channel for contractors to view these updates.</t>
+  </si>
+  <si>
+    <t>200-300 TSB access events.</t>
+  </si>
+  <si>
+    <t>Daikin App Store to integrate – Skyport App</t>
+  </si>
+  <si>
+    <t>Provide access to the Skyport App throught the Daikin Tech Hub app.</t>
+  </si>
+  <si>
+    <t>Plan is to provide all need app at one place for Technicla Service team.</t>
+  </si>
+  <si>
+    <t>NA (As per 05/04 updates, this project is likey to go to the low priority).</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Integration of Daikin Ai as a chatbot</t>
+  </si>
+  <si>
+    <t>Replace current DTH Chatbot with Daikin AI Chatbot . This will save our customers time and is the most effective way to utilize our in-house AI knowledge base.</t>
+  </si>
+  <si>
+    <t>Provide access of Artificial Integlligence acces to daikin contractors.</t>
+  </si>
+  <si>
+    <t>At least 1000 events per year.</t>
+  </si>
+  <si>
+    <t>Use OCR feature to scan serial numbers for Warranty Express</t>
+  </si>
+  <si>
+    <t>Improve the Warranty Express feature by incorporating OCR technology to scan serial numbers and automatically populate them for warranty lookup and registration.</t>
+  </si>
+  <si>
+    <t>This will create a much smoother user experience, since manually entering long serial numbers can be cumbersome and easily be incorrect inputted.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Deep linking of Matchup Xpress</t>
+  </si>
+  <si>
+    <t>Providing access of MatchupXpress using the Daikin Tech Hub app.</t>
+  </si>
+  <si>
+    <t>Provide easy access of other digital tools through the Daikin Tech Hub app.</t>
+  </si>
+  <si>
+    <t>100-200 events.</t>
+  </si>
+  <si>
+    <t>AR measurement module, Leveling module, Vibration diagnostics tool</t>
+  </si>
+  <si>
+    <t>These tool will assist technicians during installation.and diagnosis which also enhances system performance, longevity and avoid callbacks due to improper setup.</t>
+  </si>
+  <si>
+    <t>Plan is to encorporate few more tools in Daikin Tech Hub app.</t>
+  </si>
+  <si>
+    <t>Not available</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -390,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -417,6 +511,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -752,6 +849,298 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06160AE6-7A5D-E946-AABB-337BD446D968}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5" style="1" customWidth="1"/>
+    <col min="10" max="10" width="19" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A2" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" s="1" customFormat="1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" s="1" customFormat="1" ht="128" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" s="1" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+    </row>
+    <row r="6" spans="1:12" ht="64" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+    </row>
+    <row r="7" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="64" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D9DC4A3-363E-6D4C-9407-CFA72217C9BD}">
   <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1070,7 +1459,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FB2B4E7-8E64-684E-BA5C-879C72DD8766}">
   <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>